<commit_message>
fixes to tailwind 3 - 4 updates
</commit_message>
<xml_diff>
--- a/tests/assets/odk-example-form-1.xlsx
+++ b/tests/assets/odk-example-form-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dave/Sites/holpa-platform/tests/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dave/Sites/groundswell_platform/tests/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB81FD9B-2434-8C4F-A39B-C19E702624DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6481690-A88E-C040-8A61-1D620ED50A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29860" yWindow="-28300" windowWidth="37580" windowHeight="28300" tabRatio="321" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-28200" windowWidth="37580" windowHeight="28200" tabRatio="321" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -105,9 +105,6 @@
     <t>list_name</t>
   </si>
   <si>
-    <t>media::image</t>
-  </si>
-  <si>
     <t>default_language</t>
   </si>
   <si>
@@ -439,6 +436,9 @@
   </si>
   <si>
     <t>filter2</t>
+  </si>
+  <si>
+    <t>media::image::English (en)</t>
   </si>
 </sst>
 </file>
@@ -1346,7 +1346,7 @@
   <sheetData>
     <row r="1" spans="1:15" s="15" customFormat="1" ht="38" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1" s="15" t="s">
         <v>0</v>
@@ -1355,10 +1355,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" s="17" t="s">
         <v>99</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>100</v>
       </c>
       <c r="F1" s="15" t="s">
         <v>2</v>
@@ -1376,7 +1376,7 @@
         <v>4</v>
       </c>
       <c r="K1" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L1" s="15" t="s">
         <v>6</v>
@@ -1385,7 +1385,7 @@
         <v>18</v>
       </c>
       <c r="N1" s="20" t="s">
-        <v>20</v>
+        <v>131</v>
       </c>
       <c r="O1" s="18" t="s">
         <v>8</v>
@@ -1393,16 +1393,16 @@
     </row>
     <row r="2" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E2" s="11"/>
       <c r="H2" s="8"/>
@@ -1412,19 +1412,19 @@
     </row>
     <row r="3" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H3" s="8"/>
       <c r="K3" s="9"/>
@@ -1433,19 +1433,19 @@
     </row>
     <row r="4" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H4" s="8"/>
       <c r="K4" s="9"/>
@@ -1454,16 +1454,16 @@
     </row>
     <row r="5" spans="1:15" s="7" customFormat="1" ht="35" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>108</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>109</v>
       </c>
       <c r="E5" s="11"/>
       <c r="H5" s="8"/>
@@ -1473,105 +1473,105 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6" s="12" t="s">
         <v>26</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="F7" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="23" t="s">
         <v>32</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>33</v>
       </c>
       <c r="E9" s="24"/>
       <c r="F9" s="23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G9" s="23"/>
       <c r="N9" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="23" t="s">
         <v>34</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>35</v>
       </c>
       <c r="E10" s="24"/>
       <c r="F10" s="23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K10" s="4">
         <v>5</v>
@@ -1579,150 +1579,150 @@
     </row>
     <row r="11" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="26" t="s">
+      <c r="E11" s="26" t="s">
         <v>42</v>
-      </c>
-      <c r="E11" s="26" t="s">
-        <v>43</v>
       </c>
       <c r="F11" s="23"/>
       <c r="G11" s="23"/>
     </row>
     <row r="12" spans="1:15" ht="20" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E12" s="26"/>
       <c r="F12" s="23"/>
       <c r="G12" s="23"/>
       <c r="M12" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="25" t="s">
         <v>67</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>68</v>
       </c>
       <c r="D13" s="26"/>
       <c r="E13" s="26"/>
       <c r="F13" s="23"/>
       <c r="G13" s="23"/>
       <c r="I13" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="25" t="s">
         <v>63</v>
-      </c>
-      <c r="C14" s="25" t="s">
-        <v>64</v>
       </c>
       <c r="D14" s="26"/>
       <c r="E14" s="26"/>
       <c r="F14" s="23"/>
       <c r="G14" s="23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D15" s="26"/>
       <c r="E15" s="26"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
       <c r="I15" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="40" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E16" s="26"/>
       <c r="F16" s="23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G16" s="23"/>
     </row>
     <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="E17" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="26" t="s">
-        <v>84</v>
-      </c>
       <c r="F17" s="23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="20" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E18" s="26"/>
       <c r="F18" s="23"/>
@@ -1730,34 +1730,34 @@
     </row>
     <row r="19" spans="1:7" ht="80" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C19" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="26" t="s">
-        <v>122</v>
-      </c>
       <c r="E19" s="26" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G19" s="23"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D20" s="26"/>
       <c r="E20" s="26"/>
@@ -1766,13 +1766,13 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D21" s="26"/>
       <c r="E21" s="26"/>
@@ -1781,13 +1781,13 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D22" s="26"/>
       <c r="E22" s="26"/>
@@ -1799,19 +1799,19 @@
         <v>13</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C23" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="E23" s="24" t="s">
-        <v>49</v>
-      </c>
       <c r="F23" s="23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G23" s="23"/>
     </row>
@@ -1820,22 +1820,22 @@
         <v>13</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D24" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E24" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="F24" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="G24" s="23" t="s">
         <v>51</v>
-      </c>
-      <c r="F24" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="G24" s="23" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1843,16 +1843,16 @@
         <v>13</v>
       </c>
       <c r="B25" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="D25" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="D25" s="23" t="s">
-        <v>46</v>
-      </c>
       <c r="E25" s="24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F25" s="23"/>
       <c r="G25" s="23"/>
@@ -1862,16 +1862,16 @@
         <v>13</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C26" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="D26" s="23" t="s">
+      <c r="E26" s="24" t="s">
         <v>57</v>
-      </c>
-      <c r="E26" s="24" t="s">
-        <v>58</v>
       </c>
       <c r="F26" s="23"/>
       <c r="G26" s="23"/>
@@ -1949,7 +1949,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="13" customFormat="1" ht="38" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>19</v>
@@ -1958,46 +1958,46 @@
         <v>1</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" s="14">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C4" s="14">
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2005,16 +2005,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" t="s">
         <v>112</v>
-      </c>
-      <c r="D7" t="s">
-        <v>113</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -2022,16 +2022,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" t="s">
         <v>114</v>
-      </c>
-      <c r="D8" t="s">
-        <v>115</v>
       </c>
       <c r="E8">
         <v>3</v>
@@ -2039,16 +2039,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -2056,16 +2056,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C10" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="D10" t="s">
         <v>118</v>
-      </c>
-      <c r="D10" t="s">
-        <v>119</v>
       </c>
       <c r="E10">
         <v>5</v>
@@ -2079,57 +2079,57 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B13" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B14" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B15" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B16" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -2164,22 +2164,22 @@
         <v>17</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D2" s="27">
         <f ca="1">NOW()</f>
-        <v>45660.698740277781</v>
+        <v>46197.612825925928</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix 3 test results - TextSize ref; fix example form to match test expectation
</commit_message>
<xml_diff>
--- a/tests/assets/odk-example-form-1.xlsx
+++ b/tests/assets/odk-example-form-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dave/Sites/groundswell_platform/tests/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6481690-A88E-C040-8A61-1D620ED50A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F021B48-3B6E-B545-AF0E-ED5C15500AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-28200" windowWidth="37580" windowHeight="28200" tabRatio="321" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-17740" yWindow="-26120" windowWidth="37580" windowHeight="28200" tabRatio="321" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">survey!$B$1:$O$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">survey!$B$1:$N$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="130">
   <si>
     <t>type</t>
   </si>
@@ -348,9 +348,6 @@
     <t>constraint_message::English (en)</t>
   </si>
   <si>
-    <t>coffee.png</t>
-  </si>
-  <si>
     <t>English (en)</t>
   </si>
   <si>
@@ -436,9 +433,6 @@
   </si>
   <si>
     <t>filter2</t>
-  </si>
-  <si>
-    <t>media::image::English (en)</t>
   </si>
 </sst>
 </file>
@@ -727,7 +721,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
@@ -764,9 +758,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1325,7 +1316,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.6640625" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.6640625" style="1"/>
@@ -1339,14 +1330,13 @@
     <col min="11" max="11" width="24" style="4" customWidth="1"/>
     <col min="12" max="12" width="18.5" style="1" customWidth="1"/>
     <col min="13" max="13" width="18.5" style="2" customWidth="1"/>
-    <col min="14" max="14" width="18.5" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.5" style="4" customWidth="1"/>
-    <col min="16" max="16384" width="17.6640625" style="1"/>
+    <col min="14" max="14" width="18.5" style="4" customWidth="1"/>
+    <col min="15" max="16384" width="17.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="15" customFormat="1" ht="38" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="15" customFormat="1" ht="38" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1" s="15" t="s">
         <v>0</v>
@@ -1384,16 +1374,13 @@
       <c r="M1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="N1" s="20" t="s">
-        <v>131</v>
-      </c>
-      <c r="O1" s="18" t="s">
+      <c r="N1" s="18" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>12</v>
@@ -1408,11 +1395,11 @@
       <c r="H2" s="8"/>
       <c r="K2" s="9"/>
       <c r="M2" s="10"/>
-      <c r="O2" s="9"/>
-    </row>
-    <row r="3" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="N2" s="9"/>
+    </row>
+    <row r="3" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>13</v>
@@ -1429,11 +1416,11 @@
       <c r="H3" s="8"/>
       <c r="K3" s="9"/>
       <c r="M3" s="10"/>
-      <c r="O3" s="9"/>
-    </row>
-    <row r="4" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="N3" s="9"/>
+    </row>
+    <row r="4" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>14</v>
@@ -1450,30 +1437,30 @@
       <c r="H4" s="8"/>
       <c r="K4" s="9"/>
       <c r="M4" s="10"/>
-      <c r="O4" s="9"/>
-    </row>
-    <row r="5" spans="1:15" s="7" customFormat="1" ht="35" x14ac:dyDescent="0.25">
+      <c r="N4" s="9"/>
+    </row>
+    <row r="5" spans="1:14" s="7" customFormat="1" ht="35" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>108</v>
       </c>
       <c r="E5" s="11"/>
       <c r="H5" s="8"/>
       <c r="K5" s="9"/>
       <c r="M5" s="10"/>
-      <c r="O5" s="9"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N5" s="9"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>24</v>
@@ -1482,15 +1469,15 @@
         <v>25</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>27</v>
@@ -1505,15 +1492,15 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>52</v>
@@ -1528,46 +1515,43 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="24"/>
-      <c r="F9" s="23" t="s">
+      <c r="E9" s="23"/>
+      <c r="F9" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="23"/>
-      <c r="N9" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G9" s="22"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="24"/>
-      <c r="F10" s="23" t="s">
+      <c r="E10" s="23"/>
+      <c r="F10" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="G10" s="23" t="s">
+      <c r="G10" s="22" t="s">
         <v>35</v>
       </c>
       <c r="J10" s="1" t="s">
@@ -1577,137 +1561,137 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="E11" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-    </row>
-    <row r="12" spans="1:15" ht="20" x14ac:dyDescent="0.25">
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+    </row>
+    <row r="12" spans="1:14" ht="20" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="D12" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="E12" s="26"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
+      <c r="D12" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="E12" s="25"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
       <c r="M12" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
       <c r="I13" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23" t="s">
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
       <c r="I15" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="40" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="40" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="D16" s="26" t="s">
+      <c r="D16" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="E16" s="26"/>
-      <c r="F16" s="23" t="s">
+      <c r="E16" s="25"/>
+      <c r="F16" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="G16" s="23"/>
+      <c r="G16" s="22"/>
     </row>
     <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="F17" s="23" t="s">
+      <c r="F17" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="G17" s="23" t="s">
+      <c r="G17" s="22" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1715,126 +1699,126 @@
       <c r="A18" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="25" t="s">
-        <v>119</v>
-      </c>
-      <c r="D18" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
+      <c r="C18" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="25"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
     </row>
     <row r="19" spans="1:7" ht="80" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="D19" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="D19" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="E19" s="26" t="s">
-        <v>124</v>
-      </c>
-      <c r="F19" s="23" t="s">
+      <c r="E19" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="F19" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="G19" s="23"/>
+      <c r="G19" s="22"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="25" t="s">
-        <v>119</v>
-      </c>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
+      <c r="C20" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="25" t="s">
+      <c r="C22" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="23"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="23" t="s">
+      <c r="D23" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="F23" s="23" t="s">
+      <c r="F23" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="G23" s="23"/>
+      <c r="G23" s="22"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="23" t="s">
+      <c r="D24" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="F24" s="23" t="s">
+      <c r="F24" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="G24" s="23" t="s">
+      <c r="G24" s="22" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1842,63 +1826,63 @@
       <c r="A25" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="D25" s="23" t="s">
+      <c r="D25" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="24" t="s">
-        <v>129</v>
-      </c>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
+      <c r="E25" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="23" t="s">
+      <c r="B26" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="C26" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="23" t="s">
+      <c r="D26" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -1949,19 +1933,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="13" customFormat="1" ht="38" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="B1" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="20" t="s">
         <v>98</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1990,14 +1974,14 @@
       <c r="A6" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="D6" s="22" t="s">
+      <c r="C6" s="21" t="s">
         <v>109</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>108</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2007,14 +1991,14 @@
       <c r="A7" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C7" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" t="s">
         <v>111</v>
-      </c>
-      <c r="D7" t="s">
-        <v>112</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -2024,14 +2008,14 @@
       <c r="A8" t="s">
         <v>58</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C8" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8" t="s">
         <v>113</v>
-      </c>
-      <c r="D8" t="s">
-        <v>114</v>
       </c>
       <c r="E8">
         <v>3</v>
@@ -2041,14 +2025,14 @@
       <c r="A9" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -2058,49 +2042,49 @@
       <c r="A10" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C10" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" t="s">
         <v>117</v>
-      </c>
-      <c r="D10" t="s">
-        <v>118</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B11" s="22"/>
+      <c r="B11" s="21"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B12" s="22"/>
+      <c r="B12" s="21"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="21" t="s">
         <v>93</v>
       </c>
       <c r="C13" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="21" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="21" t="s">
         <v>93</v>
       </c>
       <c r="C14" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="21" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="21" t="s">
         <v>93</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -2111,7 +2095,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="21" t="s">
         <v>93</v>
       </c>
       <c r="C16" s="14" t="s">
@@ -2122,7 +2106,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="21" t="s">
         <v>93</v>
       </c>
       <c r="C17" s="14" t="s">
@@ -2169,17 +2153,17 @@
     </row>
     <row r="2" spans="1:5" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D2" s="27">
+        <v>102</v>
+      </c>
+      <c r="D2" s="26">
         <f ca="1">NOW()</f>
-        <v>46197.612825925928</v>
+        <v>46197.653356365743</v>
       </c>
       <c r="E2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>